<commit_message>
Don't show NA as duplicates in uniqueness check
</commit_message>
<xml_diff>
--- a/tests/test-files/missing-req-values.xlsx
+++ b/tests/test-files/missing-req-values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\soils\tests\test-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E561B97-AC71-4066-9E52-D81EC835D019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11C1C95-BB7B-48B8-A016-B5337044DFCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="5" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="889" uniqueCount="448">
   <si>
     <t>year</t>
   </si>
@@ -7171,9 +7171,6 @@
       <c r="D34" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>89</v>
-      </c>
       <c r="F34" s="1" t="s">
         <v>79</v>
       </c>
@@ -7293,9 +7290,6 @@
       <c r="D35" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="F35" s="1" t="s">
         <v>79</v>
       </c>
@@ -7414,9 +7408,6 @@
       </c>
       <c r="D36" s="1" t="s">
         <v>196</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>79</v>

</xml_diff>